<commit_message>
Re-ran Bugbase pipeline using filtered mapping table that excluded controls and outgroups. Also calculated groupwise significant differences for each functional trait.
</commit_message>
<xml_diff>
--- a/Analysis/Bugbase/output/auto_threshold_values.xlsx
+++ b/Analysis/Bugbase/output/auto_threshold_values.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yifanli/Documents/PhD/Projects/gcmp_analysis_2024/Analysis/Bugbase/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77158B2A-B8A1-BF42-937E-4202842C93BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{807EBC35-3DBF-7F43-BD58-5F6E9F4E2D73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19200" yWindow="520" windowWidth="19200" windowHeight="17000" xr2:uid="{2E4937D3-450C-5A44-A03C-099099B0B7BA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="21">
   <si>
     <t>Contains_Mobile_Elements</t>
   </si>
@@ -68,9 +68,6 @@
     <t>Compartment</t>
   </si>
   <si>
-    <t>Threshold value</t>
-  </si>
-  <si>
     <t>Neutral</t>
   </si>
   <si>
@@ -101,10 +98,7 @@
     <t>M00506</t>
   </si>
   <si>
-    <t>M00507</t>
-  </si>
-  <si>
-    <t>M00508</t>
+    <t>Threshold value in "Combined" fraction</t>
   </si>
 </sst>
 </file>
@@ -494,7 +488,7 @@
   <cols>
     <col min="1" max="1" width="23.5" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23.5" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.83203125" style="1"/>
     <col min="5" max="5" width="23.5" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="10.83203125" style="1"/>
@@ -510,10 +504,10 @@
         <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -521,7 +515,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1">
         <v>0.09</v>
@@ -536,7 +530,7 @@
         <v>0</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C3" s="1">
         <v>0.09</v>
@@ -551,7 +545,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="1">
         <v>0.04</v>
@@ -566,7 +560,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C5" s="1">
         <v>0.2</v>
@@ -581,7 +575,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" s="1">
         <v>0.06</v>
@@ -596,7 +590,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C7" s="1">
         <v>0.03</v>
@@ -611,7 +605,7 @@
         <v>2</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" s="1">
         <v>0.2</v>
@@ -626,7 +620,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C9" s="1">
         <v>0.2</v>
@@ -641,7 +635,7 @@
         <v>2</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10" s="1">
         <v>0.06</v>
@@ -656,7 +650,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C11" s="1">
         <v>0.6</v>
@@ -671,7 +665,7 @@
         <v>3</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12" s="1">
         <v>0.3</v>
@@ -686,7 +680,7 @@
         <v>3</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C13" s="1">
         <v>0.2</v>
@@ -701,7 +695,7 @@
         <v>4</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C14" s="1">
         <v>0.9</v>
@@ -716,7 +710,7 @@
         <v>4</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C15" s="1">
         <v>0.7</v>
@@ -731,7 +725,7 @@
         <v>4</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C16" s="1">
         <v>0.9</v>
@@ -746,7 +740,7 @@
         <v>5</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C17" s="1">
         <v>0.7</v>
@@ -761,7 +755,7 @@
         <v>5</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C18" s="1">
         <v>0.6</v>
@@ -776,7 +770,7 @@
         <v>5</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C19" s="1">
         <v>0.7</v>
@@ -791,7 +785,7 @@
         <v>6</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C20" s="1">
         <v>0.6</v>
@@ -806,7 +800,7 @@
         <v>6</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C21" s="1">
         <v>0.6</v>
@@ -821,7 +815,7 @@
         <v>6</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C22" s="1">
         <v>0.6</v>
@@ -836,7 +830,7 @@
         <v>7</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C23" s="1">
         <v>0.3</v>
@@ -851,7 +845,7 @@
         <v>7</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C24" s="1">
         <v>0.3</v>
@@ -866,7 +860,7 @@
         <v>7</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C25" s="1">
         <v>1E-3</v>
@@ -878,10 +872,10 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C26" s="1">
         <v>1E-3</v>
@@ -893,10 +887,10 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C27" s="1">
         <v>1E-3</v>
@@ -908,10 +902,10 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C28" s="1">
         <v>1E-3</v>
@@ -923,10 +917,10 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C29" s="1">
         <v>1E-3</v>
@@ -938,10 +932,10 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C30" s="1">
         <v>1E-3</v>
@@ -953,10 +947,10 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C31" s="1">
         <v>1E-3</v>
@@ -968,10 +962,10 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C32" s="1">
         <v>1E-3</v>
@@ -983,10 +977,10 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C33" s="1">
         <v>1E-3</v>
@@ -998,10 +992,10 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C34" s="1">
         <v>1E-3</v>
@@ -1013,10 +1007,10 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C35" s="1">
         <v>1E-3</v>
@@ -1028,10 +1022,10 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C36" s="1">
         <v>1E-3</v>
@@ -1043,10 +1037,10 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C37" s="1">
         <v>1E-3</v>
@@ -1058,10 +1052,10 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C38" s="1">
         <v>1E-3</v>
@@ -1073,10 +1067,10 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C39" s="1">
         <v>1E-3</v>
@@ -1088,10 +1082,10 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C40" s="1">
         <v>1E-3</v>
@@ -1103,10 +1097,10 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C41" s="1">
         <v>0.9</v>
@@ -1118,10 +1112,10 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C42" s="1">
         <v>0.9</v>
@@ -1133,10 +1127,10 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C43" s="1">
         <v>0.9</v>

</xml_diff>